<commit_message>
D(t): fair comparison, rules N2 v2/W1/W2, 100-tool blind evaluation set
- scripts/compare_d_labels.py keeps claims separate and compares binary
  questions (affirmed by the tool / uncertain / denied at any scope); the
  earlier comparison reduced claims to one status and treated scoped
  denials as not_stated, which made 60988 execute look like a disagreement
- Claude's 30 proposals revised to the agreed rules (a service name alone is
  not network; quota or bare method+route = uncertain; W1, W2): vs Menna,
  affirmed-by-tool kappa 0.90, denied kappa 0.96; 7 real differences left
- README: label provenance (LLM-assisted human vs model vs independent
  human) and the agreed protocol
- d_eval_100_{tasneem,menna}.xlsx: 100 tools of the 400-tool sample (with a
  description, one per owner per stratum), drawn before any proposals; to be
  labelled independently by both as the human reference

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labeling/d_labels_v1/d_calibration_30_claude_proposals.xlsx
+++ b/labeling/d_labels_v1/d_calibration_30_claude_proposals.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>affirmed</t>
+          <t>uncertain</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>quota spent per call implies the tool calls the YouTube API; affirmed rather than uncertain</t>
+          <t>N2 v2: operation-linked API quota, no connection described -&gt; uncertain</t>
         </is>
       </c>
     </row>
@@ -1899,41 +1899,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>affirmed</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>remote_api</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>tool</t>
-        </is>
-      </c>
+          <t>not_stated</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>closed</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Get order history for the active Schwab account.</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>N2: Schwab is not the server's own; the user's own account is a bounded domain</t>
-        </is>
-      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3822,41 +3798,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>affirmed</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>credentials</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>tool</t>
-        </is>
-      </c>
+          <t>not_stated</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>modifying</t>
-        </is>
-      </c>
+      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>Deletes one key from the operator's encrypted credential blob</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>the blob is rewritten without the key</t>
-        </is>
-      </c>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4258,41 +4210,17 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>affirmed</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>remote_api</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>tool</t>
-        </is>
-      </c>
+          <t>not_stated</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>List kata authored by a Codewars username</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>N2: Codewars is not the server's own; any username = open entities</t>
-        </is>
-      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -6924,7 +6852,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>affirmed</t>
+          <t>uncertain</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -6956,7 +6884,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>N2: Raisely is not the server's own</t>
+          <t>N2 v2: method + route without a described call -&gt; uncertain</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8738,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>affirmed</t>
+          <t>uncertain</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -8830,7 +8758,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>additive</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="L154" t="inlineStr"/>
@@ -8844,7 +8772,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="O154" t="inlineStr"/>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>persistence alone does not establish a write</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">

</xml_diff>